<commit_message>
Update workbook to use live formulas for debt schedules and instructions
Replaces flat values in the Debt Schedule with live formulas and adds a detailed convention legend to the Instructions tab.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d8376ac3-bd85-4d49-ac00-f1b0515866bf
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/elh1MDR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Microschool_Startup.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Microschool_Startup.xlsx
@@ -1424,7 +1424,7 @@
         <v>61</v>
       </c>
       <c r="D59" s="12">
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="60" spans="3:4" x14ac:dyDescent="0.25">
@@ -1432,7 +1432,7 @@
         <v>62</v>
       </c>
       <c r="D60" s="13">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="61" spans="3:4" x14ac:dyDescent="0.25">
@@ -2365,75 +2365,75 @@
       <c r="B7" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="18" t="str">
+      <c r="C7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="18" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="D7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="18" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="E7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="18" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="F7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="18" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="G7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
+        <v>6959.80855059</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="C8" s="20" t="str">
+      <c r="C8" s="20">
         <f>C6+C7</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="20" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="D8" s="20">
         <f>D6+D7</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="20" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="E8" s="20">
         <f>E6+E7</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="20" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="F8" s="20">
         <f>F6+F7</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="20" t="str">
+        <v>6959.80855059</v>
+      </c>
+      <c r="G8" s="20">
         <f>G6+G7</f>
-        <v>0</v>
+        <v>6959.80855059</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="23" t="str">
+      <c r="C10" s="23">
         <f>IF(C8&gt;0,C4/C8,IF(C4&gt;0,99.9,0))</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="23" t="str">
+        <v>-16.26481521</v>
+      </c>
+      <c r="D10" s="23">
         <f>IF(D8&gt;0,D4/D8,IF(D4&gt;0,99.9,0))</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="23" t="str">
+        <v>-18.41142599</v>
+      </c>
+      <c r="E10" s="23">
         <f>IF(E8&gt;0,E4/E8,IF(E4&gt;0,99.9,0))</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="23" t="str">
+        <v>-16.77431246</v>
+      </c>
+      <c r="F10" s="23">
         <f>IF(F8&gt;0,F4/F8,IF(F4&gt;0,99.9,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="23" t="str">
+        <v>-24.06544623</v>
+      </c>
+      <c r="G10" s="23">
         <f>IF(G8&gt;0,G4/G8,IF(G4&gt;0,99.9,0))</f>
-        <v>0</v>
+        <v>-28.80855028</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2442,23 +2442,23 @@
       </c>
       <c r="C12" s="18">
         <f>C4-C8</f>
-        <v>-113200</v>
+        <v>-120159.80855059</v>
       </c>
       <c r="D12" s="18">
         <f>D4-D8</f>
-        <v>-128140</v>
+        <v>-135099.80855059</v>
       </c>
       <c r="E12" s="18">
         <f>E4-E8</f>
-        <v>-116746.00327273</v>
+        <v>-123705.81182332</v>
       </c>
       <c r="F12" s="18">
         <f>F4-F8</f>
-        <v>-167490.89845692</v>
+        <v>-174450.70700751</v>
       </c>
       <c r="G12" s="18">
         <f>G4-G8</f>
-        <v>-200501.99456497</v>
+        <v>-207461.80311556</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
@@ -2467,23 +2467,23 @@
       </c>
       <c r="C14" s="24">
         <f>Assumptions!D57+C12</f>
-        <v>-113200</v>
+        <v>-120159.80855059</v>
       </c>
       <c r="D14" s="24">
         <f>C14+D12</f>
-        <v>-241340</v>
+        <v>-255259.61710119</v>
       </c>
       <c r="E14" s="24">
         <f>D14+E12</f>
-        <v>-358086.00327273</v>
+        <v>-378965.42892451</v>
       </c>
       <c r="F14" s="24">
         <f>E14+F12</f>
-        <v>-525576.90172964</v>
+        <v>-553416.13593202</v>
       </c>
       <c r="G14" s="24">
         <f>F14+G12</f>
-        <v>-726078.89629461</v>
+        <v>-760877.93904758</v>
       </c>
     </row>
   </sheetData>
@@ -2651,9 +2651,9 @@
       <c r="B3" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="18" t="str">
+      <c r="C3" s="18">
         <f>Assumptions!D59</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C4" s="22">
         <f>Assumptions!D60</f>
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
@@ -2678,18 +2678,18 @@
       <c r="B6" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="26" t="str">
+      <c r="C6" s="26">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>0</v>
+        <v>6959.80855059</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="23" t="str">
+      <c r="C8" s="23">
         <f>'Cash Flow &amp; DSCR'!C10</f>
-        <v>0</v>
+        <v>-16.26481521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>